<commit_message>
selectores mejorados hasta captura de accionistas dos flujos nuevos pendientes y mejora de 2da. nacionalidad
</commit_message>
<xml_diff>
--- a/cypress/fixtures/Contacto.xlsx
+++ b/cypress/fixtures/Contacto.xlsx
@@ -74,7 +74,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -83,8 +83,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4CCCC"/>
-        <bgColor rgb="FFF4CCCC"/>
+        <fgColor rgb="FFCCCCCC"/>
+        <bgColor rgb="FFCCCCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,20 +121,20 @@
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -365,8 +371,8 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""trabajo"" &amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 3)) &amp; ""01@trabajo.com"""),"trabajo22601@trabajo.com")</f>
-        <v>trabajo22601@trabajo.com</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""trabajo"" &amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 8)) &amp; ""1@gmail.com"""),"trabajo332610001@gmail.com")</f>
+        <v>trabajo332610001@gmail.com</v>
       </c>
     </row>
     <row r="3">
@@ -374,8 +380,8 @@
         <v>3</v>
       </c>
       <c r="B3" s="4" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""personal""&amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 3)) &amp; ""01@personal.com"""),"personal22601@personal.com")</f>
-        <v>personal22601@personal.com</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""personal""&amp; (RIGHT(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), 8)) &amp; ""01@personal.com"""),"personal3326100001@personal.com")</f>
+        <v>personal3326100001@personal.com</v>
       </c>
     </row>
     <row r="4">
@@ -4404,8 +4410,8 @@
       </c>
       <c r="B2" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("RIGHT(SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """"), 9)
-&amp; ""11"""),"19973322611")</f>
-        <v>19973322611</v>
+&amp; ""11"""),"73326100011")</f>
+        <v>73326100011</v>
       </c>
       <c r="C2" s="6"/>
     </row>
@@ -4415,8 +4421,8 @@
       </c>
       <c r="B3" s="3" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("RIGHT(SUBSTITUTE(IMPORTRANGE(""1_xriSLIwwVjPl8SPQz6HpPENpfWiztH_Avw6PdiYhY8"", ""'0 Cliente'!B2""), "" "", """"), 9)
-&amp; ""12"""),"19973322612")</f>
-        <v>19973322612</v>
+&amp; ""12"""),"73326100012")</f>
+        <v>73326100012</v>
       </c>
       <c r="C3" s="7"/>
     </row>

</xml_diff>